<commit_message>
add test materials with a Greek chi2
</commit_message>
<xml_diff>
--- a/inst/test_materials/test_dir/manually_extracted_stats_testpapers.xlsx
+++ b/inst/test_materials/test_dir/manually_extracted_stats_testpapers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnuijten\Documents\statcheck\inst\test_materials\test_dir\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C2C907-0027-42D9-97A6-A7D12E34925D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79051F2-3470-4975-BAB5-5C00EE567654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F0131D80-7466-4BAC-B08E-4427A3DD0F5B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{F0131D80-7466-4BAC-B08E-4427A3DD0F5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="63">
   <si>
     <t>paper_id</t>
   </si>
@@ -204,6 +204,27 @@
   </si>
   <si>
     <t>"&lt;"</t>
+  </si>
+  <si>
+    <t>paper5_pdf</t>
+  </si>
+  <si>
+    <t>χ²(8) = 13.55, p = .094.</t>
+  </si>
+  <si>
+    <t>chi2</t>
+  </si>
+  <si>
+    <t>non-ascii character</t>
+  </si>
+  <si>
+    <t>paper5_html</t>
+  </si>
+  <si>
+    <t>Paper5_chi2.pdf</t>
+  </si>
+  <si>
+    <t>Paper5_chi2.htm</t>
   </si>
 </sst>
 </file>
@@ -278,9 +299,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -318,7 +339,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -424,7 +445,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -566,7 +587,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -574,9 +595,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D938E16-0A86-461C-A717-87A651DB7BF0}">
-  <dimension ref="A1:Z23"/>
+  <dimension ref="A1:Z25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25" bestFit="1" customWidth="1"/>
     <col min="11" max="17" width="9.140625" customWidth="1"/>
   </cols>
@@ -1552,7 +1574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -1611,7 +1633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>44</v>
       </c>
@@ -1670,7 +1692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -1726,7 +1748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -1788,7 +1810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -1847,7 +1869,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>46</v>
       </c>
@@ -1903,7 +1925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>46</v>
       </c>
@@ -1963,6 +1985,130 @@
       </c>
       <c r="Y23">
         <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" t="s">
+        <v>36</v>
+      </c>
+      <c r="H24" t="s">
+        <v>29</v>
+      </c>
+      <c r="I24" t="s">
+        <v>57</v>
+      </c>
+      <c r="K24" t="s">
+        <v>58</v>
+      </c>
+      <c r="L24">
+        <v>8</v>
+      </c>
+      <c r="N24" t="s">
+        <v>54</v>
+      </c>
+      <c r="O24">
+        <v>13.55</v>
+      </c>
+      <c r="P24" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q24">
+        <v>9.4E-2</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>0</v>
+      </c>
+      <c r="U24">
+        <v>0</v>
+      </c>
+      <c r="V24">
+        <v>0</v>
+      </c>
+      <c r="W24">
+        <v>1</v>
+      </c>
+      <c r="X24">
+        <v>0</v>
+      </c>
+      <c r="Y24">
+        <v>0</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>60</v>
+      </c>
+      <c r="B25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" t="s">
+        <v>28</v>
+      </c>
+      <c r="H25" t="s">
+        <v>29</v>
+      </c>
+      <c r="I25" t="s">
+        <v>57</v>
+      </c>
+      <c r="K25" t="s">
+        <v>58</v>
+      </c>
+      <c r="L25">
+        <v>8</v>
+      </c>
+      <c r="N25" t="s">
+        <v>54</v>
+      </c>
+      <c r="O25">
+        <v>13.55</v>
+      </c>
+      <c r="P25" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q25">
+        <v>9.4E-2</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
+      <c r="T25">
+        <v>0</v>
+      </c>
+      <c r="U25">
+        <v>0</v>
+      </c>
+      <c r="V25">
+        <v>0</v>
+      </c>
+      <c r="W25">
+        <v>1</v>
+      </c>
+      <c r="X25">
+        <v>0</v>
+      </c>
+      <c r="Y25">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>